<commit_message>
Added NPS class for National Pension Scheme\
</commit_message>
<xml_diff>
--- a/BharatFinTrack/base_data/base_equity_index.xlsx
+++ b/BharatFinTrack/base_data/base_equity_index.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Debasish\Documents\coding\pypi_own\pypi_BharatFinTrack\BharatFinTrack\index_base\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Debasish\Documents\coding\pypi_own\pypi_BharatFinTrack\BharatFinTrack\base_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA876C15-2549-4067-8E6E-85AC6A653599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C4A741-B5FA-4018-ACC9-61E68E1D9A4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
Add API support for newly introduced NSE equity indices
</commit_message>
<xml_diff>
--- a/BharatFinTrack/base_data/base_equity_index.xlsx
+++ b/BharatFinTrack/base_data/base_equity_index.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Debasish\Documents\coding\pypi_own\pypi_BharatFinTrack\BharatFinTrack\base_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79C4A741-B5FA-4018-ACC9-61E68E1D9A4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6793EC24-7838-4FEC-B2FD-99BA70C708FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="188">
   <si>
     <t>NIFTY 50</t>
   </si>
@@ -538,6 +538,69 @@
   </si>
   <si>
     <t>NIFTY500 HEALTHCARE</t>
+  </si>
+  <si>
+    <t>NIFTY TOTAL MARKET MOMENTUM QUALITY 50</t>
+  </si>
+  <si>
+    <t>NIFTY SUGAR &amp; ETHANOL</t>
+  </si>
+  <si>
+    <t>NIFTY TELECOMMUNICATIONS</t>
+  </si>
+  <si>
+    <t>NIFTY CAPITAL GOODS</t>
+  </si>
+  <si>
+    <t>NIFTY RETAIL</t>
+  </si>
+  <si>
+    <t>NIFTY INSURANCE</t>
+  </si>
+  <si>
+    <t>NIFTY POWER</t>
+  </si>
+  <si>
+    <t>NIFTY HOSPITALS</t>
+  </si>
+  <si>
+    <t>NIFTY CONSUMER SERVICES</t>
+  </si>
+  <si>
+    <t>NIFTY HOUSING FINANCE</t>
+  </si>
+  <si>
+    <t>NIFTY CONSTRUCTION</t>
+  </si>
+  <si>
+    <t>NIFTY CEMENT</t>
+  </si>
+  <si>
+    <t>NIFTY COMMERCIAL &amp; TRANSPORT SERVICES</t>
+  </si>
+  <si>
+    <t>NIFTY NBFC</t>
+  </si>
+  <si>
+    <t>NIFTY REITS &amp; REALTY</t>
+  </si>
+  <si>
+    <t>NIFTY CONGLOMERATE 50</t>
+  </si>
+  <si>
+    <t>NIFTY INDIA INFRASTRUCTURE &amp; LOGISTICS</t>
+  </si>
+  <si>
+    <t>NIFTY SMALL FINANCE BANKS &amp; MICROFINANCE INSTITUTIONS</t>
+  </si>
+  <si>
+    <t>NIFTY SMALLCAP 500</t>
+  </si>
+  <si>
+    <t>NIFTY MIDSMALLCAP400 50:50</t>
+  </si>
+  <si>
+    <t>NIFTY INDIA FPI 150</t>
   </si>
 </sst>
 </file>
@@ -962,7 +1025,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B7F3278-13F7-4EB9-B476-BEA388315033}">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="45.6640625" style="1" customWidth="1"/>
@@ -1154,7 +1217,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>7</v>
+        <v>186</v>
       </c>
       <c r="B14" s="4">
         <v>38443</v>
@@ -1163,12 +1226,12 @@
         <v>1000</v>
       </c>
       <c r="D14" t="s">
-        <v>7</v>
+        <v>186</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B15" s="4">
         <v>38443</v>
@@ -1177,12 +1240,12 @@
         <v>1000</v>
       </c>
       <c r="D15" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B16" s="4">
         <v>38443</v>
@@ -1191,12 +1254,12 @@
         <v>1000</v>
       </c>
       <c r="D16" t="s">
-        <v>137</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>100</v>
+        <v>185</v>
       </c>
       <c r="B17" s="4">
         <v>38443</v>
@@ -1205,12 +1268,12 @@
         <v>1000</v>
       </c>
       <c r="D17" t="s">
-        <v>100</v>
+        <v>185</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B18" s="4">
         <v>38443</v>
@@ -1219,24 +1282,70 @@
         <v>1000</v>
       </c>
       <c r="D18" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B19" s="4">
+        <v>38443</v>
+      </c>
+      <c r="C19">
+        <v>1000</v>
+      </c>
+      <c r="D19" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" s="4">
+        <v>38443</v>
+      </c>
+      <c r="C20">
+        <v>1000</v>
+      </c>
+      <c r="D20" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B19" s="4">
+      <c r="B21" s="4">
         <v>38628</v>
       </c>
-      <c r="C19">
-        <v>1000</v>
-      </c>
-      <c r="D19" t="s">
+      <c r="C21">
+        <v>1000</v>
+      </c>
+      <c r="D21" t="s">
         <v>130</v>
       </c>
     </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="B22" s="4">
+        <v>44837</v>
+      </c>
+      <c r="C22">
+        <v>1000</v>
+      </c>
+      <c r="D22" t="s">
+        <v>187</v>
+      </c>
+    </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D22">
+    <sortCondition ref="B2:B22"/>
+    <sortCondition ref="A2:A22"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
@@ -1244,7 +1353,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40.6640625" style="1" customWidth="1"/>
@@ -1422,7 +1531,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="B13" s="3">
         <v>38443</v>
@@ -1431,12 +1540,12 @@
         <v>1000</v>
       </c>
       <c r="D13" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>76</v>
+        <v>178</v>
       </c>
       <c r="B14" s="3">
         <v>38443</v>
@@ -1444,13 +1553,13 @@
       <c r="C14">
         <v>1000</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>116</v>
+      <c r="D14" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>78</v>
+        <v>161</v>
       </c>
       <c r="B15" s="3">
         <v>38443</v>
@@ -1459,12 +1568,12 @@
         <v>1000</v>
       </c>
       <c r="D15" t="s">
-        <v>78</v>
+        <v>161</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>79</v>
+        <v>179</v>
       </c>
       <c r="B16" s="3">
         <v>38443</v>
@@ -1473,12 +1582,12 @@
         <v>1000</v>
       </c>
       <c r="D16" t="s">
-        <v>79</v>
+        <v>179</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>80</v>
+        <v>177</v>
       </c>
       <c r="B17" s="3">
         <v>38443</v>
@@ -1487,12 +1596,12 @@
         <v>1000</v>
       </c>
       <c r="D17" t="s">
-        <v>132</v>
+        <v>177</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B18" s="3">
         <v>38443</v>
@@ -1500,13 +1609,13 @@
       <c r="C18">
         <v>1000</v>
       </c>
-      <c r="D18" t="s">
-        <v>81</v>
+      <c r="D18" s="1" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B19" s="3">
         <v>38443</v>
@@ -1515,12 +1624,12 @@
         <v>1000</v>
       </c>
       <c r="D19" t="s">
-        <v>133</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>166</v>
+        <v>79</v>
       </c>
       <c r="B20" s="3">
         <v>38443</v>
@@ -1529,50 +1638,232 @@
         <v>1000</v>
       </c>
       <c r="D20" t="s">
-        <v>166</v>
+        <v>79</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="B21" s="3">
-        <v>38716</v>
+        <v>38443</v>
       </c>
       <c r="C21">
         <v>1000</v>
       </c>
       <c r="D21" t="s">
-        <v>69</v>
+        <v>132</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
+        <v>81</v>
+      </c>
+      <c r="B22" s="3">
+        <v>38443</v>
+      </c>
+      <c r="C22">
+        <v>1000</v>
+      </c>
+      <c r="D22" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>180</v>
+      </c>
+      <c r="B23" s="3">
+        <v>38443</v>
+      </c>
+      <c r="C23">
+        <v>1000</v>
+      </c>
+      <c r="D23" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>77</v>
+      </c>
+      <c r="B24" s="3">
+        <v>38443</v>
+      </c>
+      <c r="C24">
+        <v>1000</v>
+      </c>
+      <c r="D24" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>173</v>
+      </c>
+      <c r="B25" s="3">
+        <v>38443</v>
+      </c>
+      <c r="C25">
+        <v>1000</v>
+      </c>
+      <c r="D25" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>169</v>
+      </c>
+      <c r="B26" s="3">
+        <v>38443</v>
+      </c>
+      <c r="C26">
+        <v>1000</v>
+      </c>
+      <c r="D26" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>166</v>
+      </c>
+      <c r="B27" s="3">
+        <v>38443</v>
+      </c>
+      <c r="C27">
+        <v>1000</v>
+      </c>
+      <c r="D27" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>69</v>
+      </c>
+      <c r="B28" s="3">
+        <v>38716</v>
+      </c>
+      <c r="C28">
+        <v>1000</v>
+      </c>
+      <c r="D28" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
         <v>74</v>
       </c>
-      <c r="B22" s="3">
+      <c r="B29" s="3">
         <v>39080</v>
       </c>
-      <c r="C22">
-        <v>1000</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="C29">
+        <v>1000</v>
+      </c>
+      <c r="D29" t="s">
         <v>74</v>
       </c>
     </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>176</v>
+      </c>
+      <c r="B30" s="3">
+        <v>43192</v>
+      </c>
+      <c r="C30">
+        <v>1000</v>
+      </c>
+      <c r="D30" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>171</v>
+      </c>
+      <c r="B31" s="3">
+        <v>43192</v>
+      </c>
+      <c r="C31">
+        <v>1000</v>
+      </c>
+      <c r="D31" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>172</v>
+      </c>
+      <c r="B32" s="3">
+        <v>43735</v>
+      </c>
+      <c r="C32">
+        <v>1000</v>
+      </c>
+      <c r="D32" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>175</v>
+      </c>
+      <c r="B33" s="3">
+        <v>44013</v>
+      </c>
+      <c r="C33">
+        <v>1000</v>
+      </c>
+      <c r="D33" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>174</v>
+      </c>
+      <c r="B34" s="3">
+        <v>44286</v>
+      </c>
+      <c r="C34">
+        <v>1000</v>
+      </c>
+      <c r="D34" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>181</v>
+      </c>
+      <c r="B35" s="3">
+        <v>44378</v>
+      </c>
+      <c r="C35">
+        <v>1000</v>
+      </c>
+      <c r="D35" t="s">
+        <v>181</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D22">
-    <sortCondition ref="B2:B22"/>
-    <sortCondition ref="A2:A22"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D35">
+    <sortCondition ref="B2:B35"/>
+    <sortCondition ref="A2:A35"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{466D5EDC-7427-4A89-B90E-E56187B74B61}">
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="55.6640625" style="1" customWidth="1"/>
@@ -1680,7 +1971,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>84</v>
+        <v>182</v>
       </c>
       <c r="B8" s="3">
         <v>38443</v>
@@ -1688,13 +1979,13 @@
       <c r="C8">
         <v>1000</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>84</v>
+      <c r="D8" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>39</v>
+        <v>84</v>
       </c>
       <c r="B9" s="3">
         <v>38443</v>
@@ -1703,12 +1994,12 @@
         <v>1000</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>39</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>96</v>
+        <v>39</v>
       </c>
       <c r="B10" s="3">
         <v>38443</v>
@@ -1717,12 +2008,12 @@
         <v>1000</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>96</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B11" s="3">
         <v>38443</v>
@@ -1731,12 +2022,12 @@
         <v>1000</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B12" s="3">
         <v>38443</v>
@@ -1745,12 +2036,12 @@
         <v>1000</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B13" s="3">
         <v>38443</v>
@@ -1759,12 +2050,12 @@
         <v>1000</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>123</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>37</v>
+        <v>93</v>
       </c>
       <c r="B14" s="3">
         <v>38443</v>
@@ -1773,12 +2064,12 @@
         <v>1000</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B15" s="3">
         <v>38443</v>
@@ -1787,12 +2078,12 @@
         <v>1000</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>152</v>
+        <v>183</v>
       </c>
       <c r="B16" s="3">
         <v>38443</v>
@@ -1800,13 +2091,13 @@
       <c r="C16">
         <v>1000</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>152</v>
+      <c r="D16" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>153</v>
+        <v>34</v>
       </c>
       <c r="B17" s="3">
         <v>38443</v>
@@ -1814,13 +2105,13 @@
       <c r="C17">
         <v>1000</v>
       </c>
-      <c r="D17" t="s">
-        <v>153</v>
+      <c r="D17" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>102</v>
+        <v>152</v>
       </c>
       <c r="B18" s="3">
         <v>38443</v>
@@ -1829,12 +2120,12 @@
         <v>1000</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>102</v>
+        <v>152</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>41</v>
+        <v>153</v>
       </c>
       <c r="B19" s="3">
         <v>38443</v>
@@ -1842,13 +2133,13 @@
       <c r="C19">
         <v>1000</v>
       </c>
-      <c r="D19" s="1" t="s">
-        <v>41</v>
+      <c r="D19" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>36</v>
+        <v>102</v>
       </c>
       <c r="B20" s="3">
         <v>38443</v>
@@ -1857,12 +2148,12 @@
         <v>1000</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>36</v>
+        <v>102</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B21" s="3">
         <v>38443</v>
@@ -1871,12 +2162,12 @@
         <v>1000</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>105</v>
+        <v>36</v>
       </c>
       <c r="B22" s="3">
         <v>38443</v>
@@ -1885,12 +2176,12 @@
         <v>1000</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>105</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B23" s="3">
         <v>38443</v>
@@ -1899,12 +2190,12 @@
         <v>1000</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>162</v>
+        <v>105</v>
       </c>
       <c r="B24" s="3">
         <v>38443</v>
@@ -1913,12 +2204,12 @@
         <v>1000</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>162</v>
+        <v>105</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>92</v>
+        <v>40</v>
       </c>
       <c r="B25" s="3">
         <v>38443</v>
@@ -1927,12 +2218,12 @@
         <v>1000</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>145</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>91</v>
+        <v>162</v>
       </c>
       <c r="B26" s="3">
         <v>38443</v>
@@ -1941,82 +2232,82 @@
         <v>1000</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>146</v>
+        <v>162</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="B27" s="3">
-        <v>38719</v>
+        <v>38443</v>
       </c>
       <c r="C27">
         <v>1000</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>122</v>
+        <v>145</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>28</v>
+        <v>91</v>
       </c>
       <c r="B28" s="3">
-        <v>39080</v>
+        <v>38443</v>
       </c>
       <c r="C28">
         <v>1000</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>28</v>
+        <v>146</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="B29" s="3">
-        <v>39080</v>
+        <v>38719</v>
       </c>
       <c r="C29">
         <v>1000</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>29</v>
+        <v>122</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="B30" s="3">
-        <v>39814</v>
+        <v>39080</v>
       </c>
       <c r="C30">
         <v>1000</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B31" s="3">
-        <v>39814</v>
+        <v>39080</v>
       </c>
       <c r="C31">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>129</v>
+        <v>29</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B32" s="3">
         <v>39814</v>
@@ -2025,190 +2316,246 @@
         <v>1000</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B33" s="3">
         <v>39814</v>
       </c>
       <c r="C33">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B34" s="3">
-        <v>40634</v>
+        <v>39814</v>
       </c>
       <c r="C34">
         <v>1000</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B35" s="3">
-        <v>40634</v>
+        <v>39814</v>
       </c>
       <c r="C35">
         <v>1000</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>31</v>
+        <v>140</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B36" s="3">
-        <v>41640</v>
+        <v>40634</v>
       </c>
       <c r="C36">
         <v>1000</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>139</v>
+        <v>32</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B37" s="3">
-        <v>42705</v>
+        <v>40634</v>
       </c>
       <c r="C37">
         <v>1000</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>104</v>
+        <v>33</v>
       </c>
       <c r="B38" s="3">
-        <v>42737</v>
+        <v>41640</v>
       </c>
       <c r="C38">
         <v>1000</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>104</v>
+        <v>139</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>97</v>
+        <v>30</v>
       </c>
       <c r="B39" s="3">
-        <v>43192</v>
+        <v>42705</v>
       </c>
       <c r="C39">
         <v>1000</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>97</v>
+        <v>30</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>38</v>
+        <v>104</v>
       </c>
       <c r="B40" s="3">
-        <v>43192</v>
+        <v>42737</v>
       </c>
       <c r="C40">
         <v>1000</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>38</v>
+        <v>104</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="B41" s="3">
-        <v>43556</v>
+        <v>43192</v>
       </c>
       <c r="C41">
         <v>1000</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>83</v>
+        <v>38</v>
       </c>
       <c r="B42" s="3">
-        <v>43647</v>
+        <v>43192</v>
       </c>
       <c r="C42">
         <v>1000</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>83</v>
+        <v>38</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>154</v>
+        <v>107</v>
       </c>
       <c r="B43" s="3">
-        <v>44287</v>
+        <v>43556</v>
       </c>
       <c r="C43">
         <v>1000</v>
       </c>
-      <c r="D43" t="s">
-        <v>154</v>
+      <c r="D43" s="1" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B44" s="3">
+        <v>43647</v>
+      </c>
+      <c r="C44">
+        <v>1000</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B45" s="3">
+        <v>44286</v>
+      </c>
+      <c r="C45">
+        <v>1000</v>
+      </c>
+      <c r="D45" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B46" s="3">
+        <v>44286</v>
+      </c>
+      <c r="C46">
+        <v>1000</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B47" s="3">
+        <v>44287</v>
+      </c>
+      <c r="C47">
+        <v>1000</v>
+      </c>
+      <c r="D47" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B44" s="3">
+      <c r="B48" s="3">
         <v>44470</v>
       </c>
-      <c r="C44">
-        <v>1000</v>
-      </c>
-      <c r="D44" t="s">
+      <c r="C48">
+        <v>1000</v>
+      </c>
+      <c r="D48" t="s">
         <v>160</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D44">
-    <sortCondition ref="B2:B44"/>
-    <sortCondition ref="A2:A44"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D48">
+    <sortCondition ref="B2:B48"/>
+    <sortCondition ref="A2:A48"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{898D7280-DA99-43BB-B8CC-2B757AFDF5E9}">
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="45.6640625" style="1" customWidth="1"/>
@@ -2470,7 +2817,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>56</v>
+        <v>167</v>
       </c>
       <c r="B19" s="4">
         <v>38443</v>
@@ -2479,82 +2826,82 @@
         <v>1000</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>56</v>
+        <v>167</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" s="4">
+        <v>38443</v>
+      </c>
+      <c r="C20">
+        <v>1000</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B20" s="4">
-        <v>38443</v>
-      </c>
-      <c r="C20">
-        <v>1000</v>
-      </c>
-      <c r="D20" s="1" t="s">
+      <c r="B21" s="4">
+        <v>38443</v>
+      </c>
+      <c r="C21">
+        <v>1000</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="5" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B21" s="4">
-        <v>38443</v>
-      </c>
-      <c r="C21">
-        <v>1000</v>
-      </c>
-      <c r="D21" s="5" t="s">
+      <c r="B22" s="4">
+        <v>38443</v>
+      </c>
+      <c r="C22">
+        <v>1000</v>
+      </c>
+      <c r="D22" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B22" s="4">
-        <v>38443</v>
-      </c>
-      <c r="C22">
-        <v>1000</v>
-      </c>
-      <c r="D22" s="1" t="s">
+      <c r="B23" s="4">
+        <v>38443</v>
+      </c>
+      <c r="C23">
+        <v>1000</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B23" s="4">
-        <v>38443</v>
-      </c>
-      <c r="C23">
-        <v>1000</v>
-      </c>
-      <c r="D23" s="5" t="s">
+      <c r="B24" s="4">
+        <v>38443</v>
+      </c>
+      <c r="C24">
+        <v>1000</v>
+      </c>
+      <c r="D24" s="5" t="s">
         <v>51</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="B24" s="4">
-        <v>38443</v>
-      </c>
-      <c r="C24">
-        <v>1000</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B25" s="4">
         <v>38443</v>
@@ -2563,12 +2910,12 @@
         <v>1000</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>158</v>
+        <v>99</v>
       </c>
       <c r="B26" s="4">
         <v>38443</v>
@@ -2576,55 +2923,55 @@
       <c r="C26">
         <v>1000</v>
       </c>
-      <c r="D26" t="s">
-        <v>159</v>
+      <c r="D26" s="1" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B27" s="4">
+        <v>38443</v>
+      </c>
+      <c r="C27">
+        <v>1000</v>
+      </c>
+      <c r="D27" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B27" s="4">
-        <v>38443</v>
-      </c>
-      <c r="C27">
-        <v>1000</v>
-      </c>
-      <c r="D27" s="1" t="s">
+      <c r="B28" s="4">
+        <v>38443</v>
+      </c>
+      <c r="C28">
+        <v>1000</v>
+      </c>
+      <c r="D28" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="5" t="s">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B28" s="4">
-        <v>38443</v>
-      </c>
-      <c r="C28">
-        <v>1000</v>
-      </c>
-      <c r="D28" s="5" t="s">
+      <c r="B29" s="4">
+        <v>38443</v>
+      </c>
+      <c r="C29">
+        <v>1000</v>
+      </c>
+      <c r="D29" s="5" t="s">
         <v>106</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="B29" s="4">
-        <v>38443</v>
-      </c>
-      <c r="C29">
-        <v>1000</v>
-      </c>
-      <c r="D29" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="B30" s="4">
         <v>38443</v>
@@ -2633,12 +2980,12 @@
         <v>1000</v>
       </c>
       <c r="D30" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>57</v>
+        <v>156</v>
       </c>
       <c r="B31" s="4">
         <v>38443</v>
@@ -2646,27 +2993,27 @@
       <c r="C31">
         <v>1000</v>
       </c>
-      <c r="D31" s="1" t="s">
-        <v>57</v>
+      <c r="D31" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" s="4">
+        <v>38443</v>
+      </c>
+      <c r="C32">
+        <v>1000</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="B32" s="4">
-        <v>38778</v>
-      </c>
-      <c r="C32">
-        <v>1000</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="7" t="s">
-        <v>150</v>
       </c>
       <c r="B33" s="4">
         <v>38778</v>
@@ -2674,13 +3021,13 @@
       <c r="C33">
         <v>1000</v>
       </c>
-      <c r="D33" s="7" t="s">
-        <v>150</v>
+      <c r="D33" s="1" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B34" s="4">
         <v>38778</v>
@@ -2689,40 +3036,40 @@
         <v>1000</v>
       </c>
       <c r="D34" s="7" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="7" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="B35" s="4">
-        <v>39356</v>
+        <v>38778</v>
       </c>
       <c r="C35">
         <v>1000</v>
       </c>
-      <c r="D35" s="1" t="s">
-        <v>117</v>
+      <c r="D35" s="7" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B36" s="4">
-        <v>39814</v>
+        <v>39356</v>
       </c>
       <c r="C36">
         <v>1000</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="B37" s="4">
         <v>39814</v>
@@ -2731,26 +3078,26 @@
         <v>1000</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>55</v>
+        <v>121</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B38" s="3">
-        <v>39905</v>
+        <v>55</v>
+      </c>
+      <c r="B38" s="4">
+        <v>39814</v>
       </c>
       <c r="C38">
         <v>1000</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>147</v>
+        <v>55</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B39" s="3">
         <v>39905</v>
@@ -2764,7 +3111,7 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B40" s="3">
         <v>39905</v>
@@ -2778,7 +3125,7 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B41" s="3">
         <v>39905</v>
@@ -2792,21 +3139,21 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B42" s="4">
-        <v>40087</v>
+        <v>88</v>
+      </c>
+      <c r="B42" s="3">
+        <v>39905</v>
       </c>
       <c r="C42">
         <v>1000</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>163</v>
+        <v>49</v>
       </c>
       <c r="B43" s="4">
         <v>40087</v>
@@ -2814,30 +3161,44 @@
       <c r="C43">
         <v>1000</v>
       </c>
-      <c r="D43" t="s">
-        <v>163</v>
+      <c r="D43" s="1" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B44" s="4">
+        <v>40087</v>
+      </c>
+      <c r="C44">
+        <v>1000</v>
+      </c>
+      <c r="D44" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B44" s="3">
+      <c r="B45" s="3">
         <v>40269</v>
       </c>
-      <c r="C44">
-        <v>1000</v>
-      </c>
-      <c r="D44" s="1" t="s">
+      <c r="C45">
+        <v>1000</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>147</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D44">
-    <sortCondition ref="B2:B44"/>
-    <sortCondition ref="A2:A44"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D45">
+    <sortCondition ref="B2:B45"/>
+    <sortCondition ref="A2:A45"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add NIFTY500 ASHIMA index
</commit_message>
<xml_diff>
--- a/BharatFinTrack/base_data/base_equity_index.xlsx
+++ b/BharatFinTrack/base_data/base_equity_index.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Debasish\Documents\coding\pypi_own\pypi_BharatFinTrack\BharatFinTrack\base_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6793EC24-7838-4FEC-B2FD-99BA70C708FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48D68566-6356-460B-B3E8-2064E87128E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="broad" sheetId="7" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="189">
   <si>
     <t>NIFTY 50</t>
   </si>
@@ -601,6 +601,9 @@
   </si>
   <si>
     <t>NIFTY INDIA FPI 150</t>
+  </si>
+  <si>
+    <t>NIFTY500 AHIMSA</t>
   </si>
 </sst>
 </file>
@@ -1863,7 +1866,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{466D5EDC-7427-4A89-B90E-E56187B74B61}">
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="55.6640625" style="1" customWidth="1"/>
@@ -2405,49 +2408,49 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>30</v>
+        <v>188</v>
       </c>
       <c r="B39" s="3">
-        <v>42705</v>
+        <v>42461</v>
       </c>
       <c r="C39">
         <v>1000</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>30</v>
+        <v>188</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>104</v>
+        <v>30</v>
       </c>
       <c r="B40" s="3">
-        <v>42737</v>
+        <v>42705</v>
       </c>
       <c r="C40">
         <v>1000</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>104</v>
+        <v>30</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="B41" s="3">
-        <v>43192</v>
+        <v>42737</v>
       </c>
       <c r="C41">
         <v>1000</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>38</v>
+        <v>97</v>
       </c>
       <c r="B42" s="3">
         <v>43192</v>
@@ -2456,54 +2459,54 @@
         <v>1000</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>38</v>
+        <v>97</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>107</v>
+        <v>38</v>
       </c>
       <c r="B43" s="3">
-        <v>43556</v>
+        <v>43192</v>
       </c>
       <c r="C43">
         <v>1000</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>107</v>
+        <v>38</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="B44" s="3">
-        <v>43647</v>
+        <v>43556</v>
       </c>
       <c r="C44">
         <v>1000</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>83</v>
+        <v>107</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>184</v>
+        <v>83</v>
       </c>
       <c r="B45" s="3">
-        <v>44286</v>
+        <v>43647</v>
       </c>
       <c r="C45">
         <v>1000</v>
       </c>
-      <c r="D45" t="s">
-        <v>184</v>
+      <c r="D45" s="1" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="B46" s="3">
         <v>44286</v>
@@ -2511,42 +2514,56 @@
       <c r="C46">
         <v>1000</v>
       </c>
-      <c r="D46" s="1" t="s">
-        <v>168</v>
+      <c r="D46" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
       <c r="B47" s="3">
-        <v>44287</v>
+        <v>44286</v>
       </c>
       <c r="C47">
         <v>1000</v>
       </c>
-      <c r="D47" t="s">
-        <v>154</v>
+      <c r="D47" s="1" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B48" s="3">
+        <v>44287</v>
+      </c>
+      <c r="C48">
+        <v>1000</v>
+      </c>
+      <c r="D48" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B48" s="3">
+      <c r="B49" s="3">
         <v>44470</v>
       </c>
-      <c r="C48">
-        <v>1000</v>
-      </c>
-      <c r="D48" t="s">
+      <c r="C49">
+        <v>1000</v>
+      </c>
+      <c r="D49" t="s">
         <v>160</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D48">
-    <sortCondition ref="B2:B48"/>
-    <sortCondition ref="A2:A48"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D49">
+    <sortCondition ref="B2:B49"/>
+    <sortCondition ref="A2:A49"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Add API support for the new NSE index in new version
</commit_message>
<xml_diff>
--- a/BharatFinTrack/base_data/base_equity_index.xlsx
+++ b/BharatFinTrack/base_data/base_equity_index.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Debasish\Documents\coding\pypi_own\pypi_BharatFinTrack\BharatFinTrack\base_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48D68566-6356-460B-B3E8-2064E87128E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1B9D29D-9A82-4E24-8A5D-C7B778E64B07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="190">
   <si>
     <t>NIFTY 50</t>
   </si>
@@ -604,6 +604,9 @@
   </si>
   <si>
     <t>NIFTY500 AHIMSA</t>
+  </si>
+  <si>
+    <t>NIFTY REITS &amp; INVITS 90:10</t>
   </si>
 </sst>
 </file>
@@ -1866,7 +1869,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{466D5EDC-7427-4A89-B90E-E56187B74B61}">
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="55.6640625" style="1" customWidth="1"/>
@@ -2548,22 +2551,36 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B49" s="3">
+        <v>44287</v>
+      </c>
+      <c r="C49">
+        <v>1000</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B49" s="3">
+      <c r="B50" s="3">
         <v>44470</v>
       </c>
-      <c r="C49">
-        <v>1000</v>
-      </c>
-      <c r="D49" t="s">
+      <c r="C50">
+        <v>1000</v>
+      </c>
+      <c r="D50" t="s">
         <v>160</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D49">
-    <sortCondition ref="B2:B49"/>
-    <sortCondition ref="A2:A49"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D50">
+    <sortCondition ref="B2:B50"/>
+    <sortCondition ref="A2:A50"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Add newly launched NSE indices
</commit_message>
<xml_diff>
--- a/BharatFinTrack/base_data/base_equity_index.xlsx
+++ b/BharatFinTrack/base_data/base_equity_index.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Debasish\Documents\coding\pypi_own\pypi_BharatFinTrack\BharatFinTrack\base_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1B9D29D-9A82-4E24-8A5D-C7B778E64B07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F95C227D-E9D1-4744-8D68-0FB7340918C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="192">
   <si>
     <t>NIFTY 50</t>
   </si>
@@ -607,6 +607,12 @@
   </si>
   <si>
     <t>NIFTY REITS &amp; INVITS 90:10</t>
+  </si>
+  <si>
+    <t>NIFTY NEXT 100</t>
+  </si>
+  <si>
+    <t>NIFTY INDIA DEFENCE EQUAL WEIGHT</t>
   </si>
 </sst>
 </file>
@@ -1031,7 +1037,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B7F3278-13F7-4EB9-B476-BEA388315033}">
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="45.6640625" style="1" customWidth="1"/>
@@ -1335,25 +1341,39 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B22" s="4">
+        <v>40452</v>
+      </c>
+      <c r="C22">
+        <v>1000</v>
+      </c>
+      <c r="D22" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="B22" s="4">
+      <c r="B23" s="4">
         <v>44837</v>
       </c>
-      <c r="C22">
-        <v>1000</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="C23">
+        <v>1000</v>
+      </c>
+      <c r="D23" t="s">
         <v>187</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D22">
-    <sortCondition ref="B2:B22"/>
-    <sortCondition ref="A2:A22"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D23">
+    <sortCondition ref="B2:B23"/>
+    <sortCondition ref="A2:A23"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1869,7 +1889,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{466D5EDC-7427-4A89-B90E-E56187B74B61}">
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="55.6640625" style="1" customWidth="1"/>
@@ -2481,49 +2501,49 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>107</v>
+        <v>191</v>
       </c>
       <c r="B44" s="3">
-        <v>43556</v>
+        <v>43192</v>
       </c>
       <c r="C44">
         <v>1000</v>
       </c>
-      <c r="D44" s="1" t="s">
-        <v>107</v>
+      <c r="D44" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="B45" s="3">
-        <v>43647</v>
+        <v>43556</v>
       </c>
       <c r="C45">
         <v>1000</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>83</v>
+        <v>107</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>184</v>
+        <v>83</v>
       </c>
       <c r="B46" s="3">
-        <v>44286</v>
+        <v>43647</v>
       </c>
       <c r="C46">
         <v>1000</v>
       </c>
-      <c r="D46" t="s">
-        <v>184</v>
+      <c r="D46" s="1" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="B47" s="3">
         <v>44286</v>
@@ -2531,27 +2551,27 @@
       <c r="C47">
         <v>1000</v>
       </c>
-      <c r="D47" s="1" t="s">
-        <v>168</v>
+      <c r="D47" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
       <c r="B48" s="3">
-        <v>44287</v>
+        <v>44286</v>
       </c>
       <c r="C48">
         <v>1000</v>
       </c>
-      <c r="D48" t="s">
-        <v>154</v>
+      <c r="D48" s="1" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>189</v>
+        <v>154</v>
       </c>
       <c r="B49" s="3">
         <v>44287</v>
@@ -2559,28 +2579,42 @@
       <c r="C49">
         <v>1000</v>
       </c>
-      <c r="D49" s="1" t="s">
-        <v>189</v>
+      <c r="D49" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B50" s="3">
+        <v>44287</v>
+      </c>
+      <c r="C50">
+        <v>1000</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B50" s="3">
+      <c r="B51" s="3">
         <v>44470</v>
       </c>
-      <c r="C50">
-        <v>1000</v>
-      </c>
-      <c r="D50" t="s">
+      <c r="C51">
+        <v>1000</v>
+      </c>
+      <c r="D51" t="s">
         <v>160</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D50">
-    <sortCondition ref="B2:B50"/>
-    <sortCondition ref="A2:A50"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D51">
+    <sortCondition ref="B2:B51"/>
+    <sortCondition ref="A2:A51"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Add the new index API
</commit_message>
<xml_diff>
--- a/BharatFinTrack/base_data/base_equity_index.xlsx
+++ b/BharatFinTrack/base_data/base_equity_index.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Debasish\Documents\coding\pypi_own\pypi_BharatFinTrack\BharatFinTrack\base_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F95C227D-E9D1-4744-8D68-0FB7340918C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AABF882-ED42-41BA-9CA4-1E0367142D1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="broad" sheetId="7" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="193">
   <si>
     <t>NIFTY 50</t>
   </si>
@@ -613,6 +613,9 @@
   </si>
   <si>
     <t>NIFTY INDIA DEFENCE EQUAL WEIGHT</t>
+  </si>
+  <si>
+    <t>NIFTY500 GROWTH 50</t>
   </si>
 </sst>
 </file>
@@ -2623,7 +2626,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{898D7280-DA99-43BB-B8CC-2B757AFDF5E9}">
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="45.6640625" style="1" customWidth="1"/>
@@ -2997,7 +3000,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>158</v>
+        <v>192</v>
       </c>
       <c r="B27" s="4">
         <v>38443</v>
@@ -3006,54 +3009,54 @@
         <v>1000</v>
       </c>
       <c r="D27" t="s">
-        <v>159</v>
+        <v>192</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B28" s="4">
+        <v>38443</v>
+      </c>
+      <c r="C28">
+        <v>1000</v>
+      </c>
+      <c r="D28" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B28" s="4">
-        <v>38443</v>
-      </c>
-      <c r="C28">
-        <v>1000</v>
-      </c>
-      <c r="D28" s="1" t="s">
+      <c r="B29" s="4">
+        <v>38443</v>
+      </c>
+      <c r="C29">
+        <v>1000</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="5" t="s">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B29" s="4">
-        <v>38443</v>
-      </c>
-      <c r="C29">
-        <v>1000</v>
-      </c>
-      <c r="D29" s="5" t="s">
+      <c r="B30" s="4">
+        <v>38443</v>
+      </c>
+      <c r="C30">
+        <v>1000</v>
+      </c>
+      <c r="D30" s="5" t="s">
         <v>106</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="B30" s="4">
-        <v>38443</v>
-      </c>
-      <c r="C30">
-        <v>1000</v>
-      </c>
-      <c r="D30" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="B31" s="4">
         <v>38443</v>
@@ -3062,12 +3065,12 @@
         <v>1000</v>
       </c>
       <c r="D31" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>57</v>
+        <v>156</v>
       </c>
       <c r="B32" s="4">
         <v>38443</v>
@@ -3075,27 +3078,27 @@
       <c r="C32">
         <v>1000</v>
       </c>
-      <c r="D32" s="1" t="s">
-        <v>57</v>
+      <c r="D32" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B33" s="4">
+        <v>38443</v>
+      </c>
+      <c r="C33">
+        <v>1000</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="B33" s="4">
-        <v>38778</v>
-      </c>
-      <c r="C33">
-        <v>1000</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="7" t="s">
-        <v>150</v>
       </c>
       <c r="B34" s="4">
         <v>38778</v>
@@ -3103,13 +3106,13 @@
       <c r="C34">
         <v>1000</v>
       </c>
-      <c r="D34" s="7" t="s">
-        <v>150</v>
+      <c r="D34" s="1" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B35" s="4">
         <v>38778</v>
@@ -3118,40 +3121,40 @@
         <v>1000</v>
       </c>
       <c r="D35" s="7" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="7" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="B36" s="4">
-        <v>39356</v>
+        <v>38778</v>
       </c>
       <c r="C36">
         <v>1000</v>
       </c>
-      <c r="D36" s="1" t="s">
-        <v>117</v>
+      <c r="D36" s="7" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B37" s="4">
-        <v>39814</v>
+        <v>39356</v>
       </c>
       <c r="C37">
         <v>1000</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="B38" s="4">
         <v>39814</v>
@@ -3160,26 +3163,26 @@
         <v>1000</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>55</v>
+        <v>121</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B39" s="3">
-        <v>39905</v>
+        <v>55</v>
+      </c>
+      <c r="B39" s="4">
+        <v>39814</v>
       </c>
       <c r="C39">
         <v>1000</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>147</v>
+        <v>55</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B40" s="3">
         <v>39905</v>
@@ -3193,7 +3196,7 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B41" s="3">
         <v>39905</v>
@@ -3207,7 +3210,7 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B42" s="3">
         <v>39905</v>
@@ -3221,21 +3224,21 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B43" s="4">
-        <v>40087</v>
+        <v>88</v>
+      </c>
+      <c r="B43" s="3">
+        <v>39905</v>
       </c>
       <c r="C43">
         <v>1000</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>163</v>
+        <v>49</v>
       </c>
       <c r="B44" s="4">
         <v>40087</v>
@@ -3243,28 +3246,42 @@
       <c r="C44">
         <v>1000</v>
       </c>
-      <c r="D44" t="s">
-        <v>163</v>
+      <c r="D44" s="1" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B45" s="4">
+        <v>40087</v>
+      </c>
+      <c r="C45">
+        <v>1000</v>
+      </c>
+      <c r="D45" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B45" s="3">
+      <c r="B46" s="3">
         <v>40269</v>
       </c>
-      <c r="C45">
-        <v>1000</v>
-      </c>
-      <c r="D45" s="1" t="s">
+      <c r="C46">
+        <v>1000</v>
+      </c>
+      <c r="D46" s="1" t="s">
         <v>147</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D45">
-    <sortCondition ref="B2:B45"/>
-    <sortCondition ref="A2:A45"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D46">
+    <sortCondition ref="B2:B46"/>
+    <sortCondition ref="A2:A46"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>